<commit_message>
fix before full dental
</commit_message>
<xml_diff>
--- a/خصومات الاسنان - مطابقة المرافق.xlsx
+++ b/خصومات الاسنان - مطابقة المرافق.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30026"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B88F941-C7E4-4A8E-951A-CB537B7F932A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D71E527-B398-4170-9B1D-C4815B48BD46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="102">
   <si>
     <t>اسم المرفق في ملف الخصومات</t>
   </si>
@@ -104,18 +104,6 @@
     <t>cmn4pktb9002xn82kha2u3u6e</t>
   </si>
   <si>
-    <t>الحكيم طبرق</t>
-  </si>
-  <si>
-    <t>غير مطابق بقاعدة البيانات ❌</t>
-  </si>
-  <si>
-    <t>غير مطابق</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
     <t>الحياة</t>
   </si>
   <si>
@@ -173,15 +161,6 @@
     <t>cmn78k17t0034nz1nkwiklngp</t>
   </si>
   <si>
-    <t>الليبية التخصصيه</t>
-  </si>
-  <si>
-    <t>الليبيه التخصصيه</t>
-  </si>
-  <si>
-    <t>الليبيه التخصيصيه</t>
-  </si>
-  <si>
     <t>المركز العصري</t>
   </si>
   <si>
@@ -236,9 +215,6 @@
     <t>سما</t>
   </si>
   <si>
-    <t>شركة بنيان الصحة للخدمات الطبية(مركز بيور سمايل)</t>
-  </si>
-  <si>
     <t>cmn4pktb8000nn82khqzbuxdd</t>
   </si>
   <si>
@@ -284,9 +260,6 @@
     <t>cmn4pktb9003on82kw9kzwrgo</t>
   </si>
   <si>
-    <t>مركز القمة</t>
-  </si>
-  <si>
     <t>مركز الليبي</t>
   </si>
   <si>
@@ -345,13 +318,16 @@
   </si>
   <si>
     <t>cmn4pktb90041n82k6rvl4qat</t>
+  </si>
+  <si>
+    <t>مركز سما للاسنان</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -371,14 +347,8 @@
       <color rgb="FF008000"/>
       <name val="Arial"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -395,11 +365,6 @@
         <fgColor rgb="FFE8F5E9"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEEEE"/>
-      </patternFill>
-    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -413,7 +378,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -425,12 +390,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -772,7 +731,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D46"/>
+  <dimension ref="A1:D41"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="30" customWidth="1"/>
@@ -925,53 +884,53 @@
       <c r="A11" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C11" s="6" t="s">
+      <c r="C11" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" s="4" t="s">
         <v>31</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="C12" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>34</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="C13" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>37</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D14" s="4" t="s">
         <v>38</v>
@@ -979,69 +938,69 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="C15" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" s="4" t="s">
         <v>41</v>
-      </c>
-      <c r="C15" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="C16" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D16" s="4" t="s">
         <v>44</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="C17" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D17" s="4" t="s">
         <v>47</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D17" s="4" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>50</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D19" s="4" t="s">
         <v>51</v>
@@ -1049,114 +1008,114 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B20" s="2" t="s">
-        <v>50</v>
-      </c>
       <c r="C20" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>41</v>
+        <v>24</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>63</v>
+        <v>101</v>
       </c>
       <c r="C25" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>24</v>
+        <v>5</v>
       </c>
       <c r="C26" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>25</v>
+        <v>7</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>67</v>
+        <v>40</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>68</v>
+        <v>41</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
@@ -1167,7 +1126,7 @@
         <v>70</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D28" s="4" t="s">
         <v>71</v>
@@ -1178,41 +1137,41 @@
         <v>72</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>7</v>
+        <v>44</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>75</v>
+      </c>
+      <c r="C31" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="D31" s="4" t="s">
         <v>76</v>
-      </c>
-      <c r="B31" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
@@ -1220,27 +1179,27 @@
         <v>77</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>78</v>
+        <v>5</v>
       </c>
       <c r="C32" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>79</v>
+        <v>7</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="D33" s="4" t="s">
         <v>80</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C33" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D33" s="4" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
@@ -1248,13 +1207,13 @@
         <v>81</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C34" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
@@ -1276,156 +1235,89 @@
         <v>85</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>5</v>
+        <v>86</v>
       </c>
       <c r="C36" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>7</v>
+        <v>87</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>87</v>
+        <v>43</v>
       </c>
       <c r="C37" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>88</v>
+        <v>44</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B38" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="C38" s="6" t="s">
-        <v>31</v>
+      <c r="B38" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>6</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>32</v>
+        <v>91</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>57</v>
+        <v>93</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>58</v>
+        <v>94</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="2" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="2" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A42" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="B42" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C42" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D42" s="4" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A43" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="B43" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="C43" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D43" s="4" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A44" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="B44" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="C44" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D44" s="4" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A45" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="C45" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="D45" s="4" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A46" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="B46" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="C46" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D46" s="4" t="s">
-        <v>109</v>
-      </c>
-    </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D42">
+    <sortCondition ref="A2:A42"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="75" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
 </worksheet>

</xml_diff>